<commit_message>
feat(test-data): seed 5000 inventory pallets + 50-vehicle outbound test data
- scripts/import_materials.js: remove old_code, storage_category, manufacturer_code
  (manufacturer now identified from QR code char 6: B=Ba Vì D=Bình Dương O=Gia công)
- scripts/seed_inventory.js: inserts 5000 InventoryEntry (2800×Ba Vì 180 + 2200×Ba Vì 110)
  across 20 locations, QA OK, all IN_STOCK, production dates Jan–Apr 2026
- scripts/gen_outbound_data.js: generates 50-vehicle Excel (20 xe pallet, 20 xe container,
  10 xe xá), ~3000 cartons/xe, total 182k cartons
- Material_Template.xlsx: regenerated without the 3 removed columns
- Outbound_Test_Data.xlsx: 50-vehicle test file ready to upload

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Material_Template.xlsx
+++ b/Material_Template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:M3"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
@@ -410,11 +410,8 @@
     <col min="9" max="9" width="12.83203125" customWidth="1"/>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
     <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="22.83203125" customWidth="1"/>
-    <col min="13" max="13" width="12.83203125" customWidth="1"/>
-    <col min="14" max="14" width="14.83203125" customWidth="1"/>
-    <col min="15" max="15" width="20.83203125" customWidth="1"/>
-    <col min="16" max="16" width="20.83203125" customWidth="1"/>
+    <col min="12" max="12" width="20.83203125" customWidth="1"/>
+    <col min="13" max="13" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -452,18 +449,9 @@
         <v>HSD (ngày)</v>
       </c>
       <c r="L1" t="str">
-        <v>Bảo quản (UHT/Fresh/Frozen)</v>
+        <v>Tên rút gọn (tuỳ chọn)</v>
       </c>
       <c r="M1" t="str">
-        <v>Mã cũ</v>
-      </c>
-      <c r="N1" t="str">
-        <v>Mã NMSX</v>
-      </c>
-      <c r="O1" t="str">
-        <v>Tên rút gọn (tuỳ chọn)</v>
-      </c>
-      <c r="P1" t="str">
         <v>Ghi chú</v>
       </c>
     </row>
@@ -502,74 +490,56 @@
         <v>shelf_life_days</v>
       </c>
       <c r="L2" t="str">
-        <v>storage_category</v>
+        <v>custom_short_name</v>
       </c>
       <c r="M2" t="str">
-        <v>old_code</v>
-      </c>
-      <c r="N2" t="str">
-        <v>manufacturer_code</v>
-      </c>
-      <c r="O2" t="str">
-        <v>custom_short_name</v>
-      </c>
-      <c r="P2" t="str">
         <v>notes</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>10010001</v>
+        <v>510000001</v>
       </c>
       <c r="B3" t="str">
-        <v>Sữa tươi TH True Milk 1L</v>
+        <v>LOF Ba Vì Sữa tươi Có đường 200mlx48</v>
       </c>
       <c r="C3" t="str">
         <v>Thành phẩm</v>
       </c>
       <c r="D3" t="str">
-        <v>Fresh</v>
+        <v>200</v>
       </c>
       <c r="E3" t="str">
         <v>thùng</v>
       </c>
       <c r="F3">
-        <v>12.5</v>
+        <v>12</v>
       </c>
       <c r="G3">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="H3">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="I3">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="J3">
-        <v>720</v>
+        <v>4800</v>
       </c>
       <c r="K3">
-        <v>30</v>
+        <v>240</v>
       </c>
       <c r="L3" t="str">
-        <v>Fresh</v>
+        <v>Ba Vì 200</v>
       </c>
       <c r="M3" t="str">
-        <v>OLD001</v>
-      </c>
-      <c r="N3" t="str">
-        <v>TH</v>
-      </c>
-      <c r="O3" t="str">
-        <v>TH 1L</v>
-      </c>
-      <c r="P3" t="str">
         <v>Hàng mẫu</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>